<commit_message>
dev: handle emtpy lines, as they may be treated as end of file
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T1.xlsx
+++ b/Ref_Files/Test_Excell_T1.xlsx
@@ -5,11 +5,10 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Prices" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">КСС_ОП1!$A$7</definedName>
@@ -24,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="55">
   <si>
     <t xml:space="preserve">Тест</t>
   </si>
@@ -229,39 +228,6 @@
   </si>
   <si>
     <t xml:space="preserve">ОБЩО ВСИЧКО В ЕВРО С ДДС (XV+XVI):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test-10</t>
   </si>
 </sst>
 </file>
@@ -991,7 +957,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
@@ -1001,7 +967,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.86"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="8" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1016,6 +983,7 @@
       </c>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
+      <c r="O1" s="0"/>
     </row>
     <row r="2" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
@@ -1029,6 +997,7 @@
       <c r="G2" s="9"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="O2" s="0"/>
     </row>
     <row r="3" s="8" customFormat="true" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
@@ -1042,6 +1011,7 @@
       <c r="G3" s="10"/>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
+      <c r="O3" s="0"/>
     </row>
     <row r="4" s="8" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12"/>
@@ -1053,6 +1023,7 @@
       <c r="G4" s="12"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
+      <c r="O4" s="0"/>
     </row>
     <row r="5" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13"/>
@@ -1064,6 +1035,7 @@
       <c r="G5" s="13"/>
       <c r="H5" s="14"/>
       <c r="I5" s="15"/>
+      <c r="O5" s="0"/>
     </row>
     <row r="6" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
@@ -1077,6 +1049,7 @@
       <c r="G6" s="16"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
+      <c r="O6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
@@ -1279,7 +1252,7 @@
       <c r="D19" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="30" t="str">
+      <c r="E19" s="30" t="n">
         <f aca="false">E18*6</f>
         <v>30</v>
       </c>
@@ -1297,7 +1270,7 @@
       <c r="D20" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="30" t="str">
+      <c r="E20" s="30" t="n">
         <f aca="false">E18*1</f>
         <v>5</v>
       </c>
@@ -1332,7 +1305,7 @@
       <c r="D22" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="30" t="str">
+      <c r="E22" s="30" t="n">
         <f aca="false">E21*6</f>
         <v>60</v>
       </c>
@@ -1525,7 +1498,7 @@
       <c r="D34" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E34" s="30" t="str">
+      <c r="E34" s="30" t="n">
         <f aca="false">E33*6</f>
         <v>30</v>
       </c>
@@ -1543,7 +1516,7 @@
       <c r="D35" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E35" s="30" t="str">
+      <c r="E35" s="30" t="n">
         <f aca="false">E33*1</f>
         <v>5</v>
       </c>
@@ -1673,7 +1646,7 @@
       <c r="D44" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E44" s="30" t="str">
+      <c r="E44" s="30" t="n">
         <f aca="false">E43*1</f>
         <v>20</v>
       </c>
@@ -1691,7 +1664,7 @@
       <c r="D45" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E45" s="30" t="str">
+      <c r="E45" s="30" t="n">
         <f aca="false">E44*6</f>
         <v>120</v>
       </c>
@@ -1927,6 +1900,7 @@
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
+      <c r="O60" s="0"/>
     </row>
     <row r="61" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="30" t="s">
@@ -1939,7 +1913,7 @@
       <c r="D61" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E61" s="30" t="str">
+      <c r="E61" s="30" t="n">
         <f aca="false">E60*6</f>
         <v>60</v>
       </c>
@@ -1952,6 +1926,7 @@
       <c r="L61" s="1"/>
       <c r="M61" s="1"/>
       <c r="N61" s="1"/>
+      <c r="O61" s="0"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="30" t="s">
@@ -1964,7 +1939,7 @@
       <c r="D62" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="E62" s="30" t="str">
+      <c r="E62" s="30" t="n">
         <f aca="false">E60*1</f>
         <v>10</v>
       </c>
@@ -1994,6 +1969,7 @@
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
       <c r="N63" s="1"/>
+      <c r="O63" s="0"/>
     </row>
     <row r="64" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="32" t="s">
@@ -2014,6 +1990,7 @@
       <c r="L64" s="1"/>
       <c r="M64" s="1"/>
       <c r="N64" s="1"/>
+      <c r="O64" s="0"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="38" t="s">
@@ -2146,433 +2123,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.86"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="25" t="n">
-        <v>1150</v>
-      </c>
-      <c r="F3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" s="25" t="n">
-        <f aca="false">E3*F3</f>
-        <v>1150</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="25" t="n">
-        <v>700</v>
-      </c>
-      <c r="F4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="25" t="n">
-        <f aca="false">E4*F4</f>
-        <v>700</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="25" t="n">
-        <v>400</v>
-      </c>
-      <c r="F5" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="25" t="n">
-        <f aca="false">E5*F5</f>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>898</v>
-      </c>
-      <c r="F6" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="25" t="n">
-        <f aca="false">E6*F6</f>
-        <v>898</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="25" t="n">
-        <v>338</v>
-      </c>
-      <c r="F7" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="25" t="n">
-        <f aca="false">E7*F7</f>
-        <v>338</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="C8" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>54</v>
-      </c>
-      <c r="F8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="25" t="n">
-        <f aca="false">E8*F8</f>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="28" t="n">
-        <v>30</v>
-      </c>
-      <c r="F9" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="25" t="n">
-        <f aca="false">E9*F9</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="30" t="n">
-        <v>180</v>
-      </c>
-      <c r="F10" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="25" t="n">
-        <f aca="false">E10*F10</f>
-        <v>180</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="30" t="n">
-        <v>30</v>
-      </c>
-      <c r="F11" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="25" t="n">
-        <f aca="false">E11*F11</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="28" t="n">
-        <v>35</v>
-      </c>
-      <c r="F12" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="25" t="n">
-        <f aca="false">E12*F12</f>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="30"/>
-      <c r="C13" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="30" t="n">
-        <v>210</v>
-      </c>
-      <c r="F13" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="25" t="n">
-        <f aca="false">E13*F13</f>
-        <v>210</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="30" t="n">
-        <v>15</v>
-      </c>
-      <c r="F14" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="25" t="n">
-        <f aca="false">E14*F14</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="25" t="n">
-        <v>92</v>
-      </c>
-      <c r="F15" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="25" t="n">
-        <f aca="false">E15*F15</f>
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="25" t="n">
-        <v>600</v>
-      </c>
-      <c r="F17" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="25" t="n">
-        <f aca="false">E17*F17</f>
-        <v>600</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="25" t="n">
-        <v>200</v>
-      </c>
-      <c r="F18" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="25" t="n">
-        <f aca="false">E18*F18</f>
-        <v>200</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A16:A17"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
dev-auto-content: added new tab with analysis
</commit_message>
<xml_diff>
--- a/Ref_Files/Test_Excell_T1.xlsx
+++ b/Ref_Files/Test_Excell_T1.xlsx
@@ -1,76 +1,88 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr filterPrivacy="1"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView activeTab="0" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="КСС_ОП1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="КСС_ОП1" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="Prices" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_Hlk165973344" vbProcedure="false">КСС_ОП1!$A$7</definedName>
+    <definedName name="_Hlk165973344" localSheetId="0" hidden="0">'КСС_ОП1'!$A$7</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="55">
-  <si>
-    <t xml:space="preserve">Тест</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Някаква информация</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Някакво по-дълго описание на поставената задача. Може да съдържа няколко реда …</t>
-  </si>
-  <si>
-    <t xml:space="preserve">КОЛИЧЕСТВЕНО - СТОЙНОСТНА СМЕТКА (КСС)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">№ по ред</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Анализи</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Наименование на работите</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ед. мярка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Колич.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ед. цена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стойност</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сецкия 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Строителна част</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00100, с два реда</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="55">
+  <si>
+    <t>Тест</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Някаква информация</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Някакво по-дълго описание на поставената задача. Може да съдържа няколко реда …</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>КОЛИЧЕСТВЕНО - СТОЙНОСТНА СМЕТКА (КСС)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>№ по ред</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Анализи</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Наименование на работите</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ед. мярка</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Колич.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ед. цена</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Стойност</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Сецкия 1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>I.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Строителна част</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00100, с два реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция Х-00100 измерване</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <r>
@@ -81,7 +93,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">m</t>
+      <t>m</t>
     </r>
     <r>
       <rPr>
@@ -92,14 +104,17 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">3</t>
+      <t>3</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00300</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00200</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00300</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <r>
@@ -110,7 +125,7 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">m</t>
+      <t>m</t>
     </r>
     <r>
       <rPr>
@@ -121,125 +136,161 @@
         <family val="1"/>
         <charset val="204"/>
       </rPr>
-      <t xml:space="preserve">2</t>
+      <t>2</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">II.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Монтажна част</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">бр.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00700</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00702</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00900</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 3:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Секция 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция 1-00100, с два реда</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>II.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Монтажна част</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00400</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>m'</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00500</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00600</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>бр.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00700</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00701</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00702</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00800</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00801</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00900</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 3:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Секция 2</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция 1-00100, с два реда</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t xml:space="preserve">      -  операция 1-00100 измерване</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 4:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Секция 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">III.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 5:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Секция 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция Х-00901</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 6:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XIV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 18:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XV.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩА СТОЙНОСТ В ЕВРО БЕЗ ДДС (I+II+III+IV+V+VI+VII+VIII+IX+X+XI+XII+XIII+XIV):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XVI.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДДС 20 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XVII.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ОБЩО ВСИЧКО В ЕВРО С ДДС (XV+XVI):</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00802</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 4:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Секция 3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>III.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 5:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Секция 4</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Операция Х-00901</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>IV.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 6:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>XIV.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩА СТОЙНОСТ СМР ВОДОПРОВОДЕН КЛОН 18:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>XV.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩА СТОЙНОСТ В ЕВРО БЕЗ ДДС (I+II+III+IV+V+VI+VII+VIII+IX+X+XI+XII+XIII+XIV):</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>XVI.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ДДС 20 %</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>XVII.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ОБЩО ВСИЧКО В ЕВРО С ДДС (XV+XVI):</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -282,35 +333,35 @@
       <charset val="204"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="16"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="204"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -318,7 +369,7 @@
       <charset val="204"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -425,56 +476,56 @@
     </fill>
   </fills>
   <borders count="8">
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left/>
       <right/>
       <top/>
       <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="medium"/>
       <right style="thin"/>
       <top style="medium"/>
       <bottom style="medium"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right/>
       <top style="medium"/>
       <bottom style="medium"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="medium"/>
       <right style="medium"/>
       <top style="medium"/>
       <bottom style="medium"/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border diagonalUp="0" diagonalDown="0">
       <left style="thin"/>
       <right/>
       <top style="thin"/>
@@ -483,230 +534,230 @@
     </border>
   </borders>
   <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="50">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="bottom" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="top" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="bottom" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="8" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="9" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="general" vertical="center" wrapText="0" textRotation="0"/>
+      <protection locked="1" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -717,71 +768,17 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF8EFD8"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0D66A"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFEAF1CD"/>
-      <rgbColor rgb="FFFFE699"/>
-      <rgbColor rgb="FF9DC3E6"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFD966"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFDEB340"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Тема на Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема на Office">
   <a:themeElements>
     <a:clrScheme name="Оffice">
       <a:dk1>
@@ -823,12 +820,12 @@
     </a:clrScheme>
     <a:fontScheme name="Оffice">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -860,7 +857,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -884,7 +881,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -944,49 +941,48 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O70"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr customHeight="0" defaultColWidth="9.14453125" defaultRowHeight="15" outlineLevelCol="0" outlineLevelRow="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="31.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.86"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="8" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="9.14"/>
+    <col min="1" max="1" width="10.14" customWidth="1" style="1"/>
+    <col min="2" max="2" width="11.36" customWidth="1" style="1"/>
+    <col min="3" max="3" width="31.32" customWidth="1" style="1"/>
+    <col min="4" max="4" width="10.71" customWidth="1" style="1"/>
+    <col min="5" max="5" width="7.86" customWidth="1" style="1"/>
+    <col min="6" max="6" width="9.43" customWidth="1" style="1"/>
+    <col min="7" max="7" width="15.86" customWidth="1" style="1"/>
+    <col min="8" max="14" width="9.14" customWidth="1" style="1"/>
+    <col min="16" max="16384" width="9.14" customWidth="1" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:15" ht="15" customHeight="1" customFormat="1" s="8">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
       <c r="D1" s="2"/>
       <c r="E1" s="4"/>
       <c r="F1" s="5"/>
-      <c r="G1" s="6" t="s">
+      <c r="G1" t="s" s="6">
         <v>0</v>
       </c>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
-      <c r="O1" s="0"/>
-    </row>
-    <row r="2" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="O1"/>
+    </row>
+    <row r="2" spans="1:15" ht="15" customHeight="1" customFormat="1" s="8">
+      <c r="A2" t="s" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="9"/>
@@ -997,10 +993,10 @@
       <c r="G2" s="9"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-      <c r="O2" s="0"/>
-    </row>
-    <row r="3" s="8" customFormat="true" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="O2"/>
+    </row>
+    <row r="3" spans="1:15" ht="54.75" customHeight="1" customFormat="1" s="8">
+      <c r="A3" t="s" s="10">
         <v>2</v>
       </c>
       <c r="B3" s="10"/>
@@ -1011,9 +1007,9 @@
       <c r="G3" s="10"/>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
-      <c r="O3" s="0"/>
-    </row>
-    <row r="4" s="8" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O3"/>
+    </row>
+    <row r="4" spans="1:15" ht="13.5" customHeight="1" customFormat="1" s="8">
       <c r="A4" s="12"/>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -1023,9 +1019,9 @@
       <c r="G4" s="12"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
-      <c r="O4" s="0"/>
-    </row>
-    <row r="5" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O4"/>
+    </row>
+    <row r="5" spans="1:15" ht="15" customFormat="1" s="8">
       <c r="A5" s="13"/>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -1035,10 +1031,10 @@
       <c r="G5" s="13"/>
       <c r="H5" s="14"/>
       <c r="I5" s="15"/>
-      <c r="O5" s="0"/>
-    </row>
-    <row r="6" s="8" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="O5"/>
+    </row>
+    <row r="6" spans="1:15" ht="15" customFormat="1" s="8">
+      <c r="A6" t="s" s="16">
         <v>3</v>
       </c>
       <c r="B6" s="16"/>
@@ -1049,33 +1045,33 @@
       <c r="G6" s="16"/>
       <c r="H6" s="17"/>
       <c r="I6" s="17"/>
-      <c r="O6" s="0"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="O6"/>
+    </row>
+    <row r="7" spans="1:7" ht="15">
+      <c r="A7" t="s" s="18">
         <v>4</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" t="s" s="18">
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" t="s" s="18">
         <v>6</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" t="s" s="18">
         <v>7</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" t="s" s="18">
         <v>8</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" t="s" s="18">
         <v>9</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" t="s" s="18">
         <v>10</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+    <row r="8" spans="1:7" ht="15">
+      <c r="A8" t="s" s="19">
         <v>11</v>
       </c>
       <c r="B8" s="19"/>
@@ -1085,12 +1081,12 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s" s="20">
         <v>12</v>
       </c>
       <c r="B9" s="20"/>
-      <c r="C9" s="21" t="s">
+      <c r="C9" t="s" s="21">
         <v>13</v>
       </c>
       <c r="D9" s="22"/>
@@ -1098,12 +1094,12 @@
       <c r="F9" s="22"/>
       <c r="G9" s="22"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" s="23">
         <v>1</v>
       </c>
       <c r="B10" s="23"/>
-      <c r="C10" s="24" t="s">
+      <c r="C10" t="s" s="24">
         <v>14</v>
       </c>
       <c r="D10" s="25"/>
@@ -1111,61 +1107,61 @@
       <c r="F10" s="25"/>
       <c r="G10" s="25"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:7" ht="15">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="26" t="s">
+      <c r="C11" t="s" s="26">
         <v>15</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" t="s" s="25">
         <v>16</v>
       </c>
-      <c r="E11" s="25" t="n">
+      <c r="E11" s="25">
         <v>200</v>
       </c>
       <c r="F11" s="25"/>
       <c r="G11" s="25"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" s="23">
         <v>2</v>
       </c>
       <c r="B12" s="23"/>
-      <c r="C12" s="27" t="s">
+      <c r="C12" t="s" s="27">
         <v>17</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" t="s" s="25">
         <v>16</v>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="E12" s="25">
         <v>100</v>
       </c>
       <c r="F12" s="25"/>
       <c r="G12" s="25"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" s="23">
         <v>3</v>
       </c>
       <c r="B13" s="23"/>
-      <c r="C13" s="27" t="s">
+      <c r="C13" t="s" s="27">
         <v>18</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" t="s" s="25">
         <v>19</v>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E13" s="25">
         <v>150</v>
       </c>
       <c r="F13" s="25"/>
       <c r="G13" s="25"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s" s="20">
         <v>20</v>
       </c>
       <c r="B14" s="20"/>
-      <c r="C14" s="21" t="s">
+      <c r="C14" t="s" s="21">
         <v>21</v>
       </c>
       <c r="D14" s="22"/>
@@ -1173,168 +1169,168 @@
       <c r="F14" s="22"/>
       <c r="G14" s="22"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="n">
+    <row r="15" spans="1:7" ht="15">
+      <c r="A15" s="25">
         <v>1</v>
       </c>
       <c r="B15" s="25"/>
-      <c r="C15" s="27" t="s">
+      <c r="C15" t="s" s="27">
         <v>22</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E15" s="25">
         <v>299</v>
       </c>
       <c r="F15" s="25"/>
       <c r="G15" s="25"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="n">
+    <row r="16" spans="1:7" ht="15">
+      <c r="A16" s="25">
         <v>2</v>
       </c>
       <c r="B16" s="25"/>
-      <c r="C16" s="27" t="s">
+      <c r="C16" t="s" s="27">
         <v>24</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="25">
         <v>119</v>
       </c>
       <c r="F16" s="25"/>
       <c r="G16" s="25"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="n">
+    <row r="17" spans="1:7" ht="15">
+      <c r="A17" s="25">
         <v>3</v>
       </c>
       <c r="B17" s="25"/>
-      <c r="C17" s="27" t="s">
+      <c r="C17" t="s" s="27">
         <v>25</v>
       </c>
-      <c r="D17" s="25" t="s">
+      <c r="D17" t="s" s="25">
         <v>26</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="25">
         <v>2</v>
       </c>
       <c r="F17" s="25"/>
       <c r="G17" s="25"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="n">
+    <row r="18" spans="1:7" ht="15">
+      <c r="A18" s="28">
         <v>4</v>
       </c>
       <c r="B18" s="28"/>
-      <c r="C18" s="29" t="s">
+      <c r="C18" t="s" s="29">
         <v>27</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" t="s" s="28">
         <v>26</v>
       </c>
-      <c r="E18" s="28" t="n">
+      <c r="E18" s="28">
         <v>5</v>
       </c>
       <c r="F18" s="28"/>
       <c r="G18" s="28"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="s">
+    <row r="19" spans="1:7" ht="15">
+      <c r="A19" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B19" s="30"/>
-      <c r="C19" s="31" t="s">
+      <c r="C19" t="s" s="31">
         <v>29</v>
       </c>
-      <c r="D19" s="30" t="s">
+      <c r="D19" t="s" s="30">
         <v>23</v>
       </c>
-      <c r="E19" s="30" t="n">
-        <f aca="false">E18*6</f>
+      <c r="E19" t="str" s="30">
+        <f>E18*6</f>
         <v>30</v>
       </c>
       <c r="F19" s="30"/>
       <c r="G19" s="30"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:7" ht="15">
+      <c r="A20" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B20" s="30"/>
-      <c r="C20" s="31" t="s">
+      <c r="C20" t="s" s="31">
         <v>30</v>
       </c>
-      <c r="D20" s="30" t="s">
+      <c r="D20" t="s" s="30">
         <v>26</v>
       </c>
-      <c r="E20" s="30" t="n">
-        <f aca="false">E18*1</f>
+      <c r="E20" t="str" s="30">
+        <f>E18*1</f>
         <v>5</v>
       </c>
       <c r="F20" s="30"/>
       <c r="G20" s="30"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="n">
+    <row r="21" spans="1:7" ht="15">
+      <c r="A21" s="28">
         <v>5</v>
       </c>
       <c r="B21" s="28"/>
-      <c r="C21" s="29" t="s">
+      <c r="C21" t="s" s="29">
         <v>31</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D21" t="s" s="28">
         <v>26</v>
       </c>
-      <c r="E21" s="28" t="n">
+      <c r="E21" s="28">
         <v>10</v>
       </c>
       <c r="F21" s="28"/>
       <c r="G21" s="28"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30" t="s">
+    <row r="22" spans="1:7" ht="15">
+      <c r="A22" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B22" s="30"/>
-      <c r="C22" s="31" t="s">
+      <c r="C22" t="s" s="31">
         <v>32</v>
       </c>
-      <c r="D22" s="30" t="s">
+      <c r="D22" t="s" s="30">
         <v>23</v>
       </c>
-      <c r="E22" s="30" t="n">
-        <f aca="false">E21*6</f>
+      <c r="E22" t="str" s="30">
+        <f>E21*6</f>
         <v>60</v>
       </c>
       <c r="F22" s="30"/>
       <c r="G22" s="30"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="n">
+    <row r="23" spans="1:7" ht="15">
+      <c r="A23" s="25">
         <v>6</v>
       </c>
       <c r="B23" s="25"/>
-      <c r="C23" s="27" t="s">
+      <c r="C23" t="s" s="27">
         <v>33</v>
       </c>
-      <c r="D23" s="25" t="s">
+      <c r="D23" t="s" s="25">
         <v>26</v>
       </c>
-      <c r="E23" s="25" t="n">
+      <c r="E23" s="25">
         <v>20</v>
       </c>
       <c r="F23" s="25"/>
       <c r="G23" s="25"/>
     </row>
-    <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
+    <row r="24" spans="1:14" ht="18.75" customHeight="1">
+      <c r="A24" t="s" s="32">
         <v>12</v>
       </c>
       <c r="B24" s="32"/>
-      <c r="C24" s="33" t="s">
+      <c r="C24" t="s" s="33">
         <v>34</v>
       </c>
       <c r="D24" s="33"/>
@@ -1348,8 +1344,8 @@
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+    <row r="25" spans="1:14" ht="15">
+      <c r="A25" t="s" s="19">
         <v>35</v>
       </c>
       <c r="B25" s="19"/>
@@ -1365,12 +1361,12 @@
       <c r="M25" s="25"/>
       <c r="N25" s="25"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+    <row r="26" spans="1:7" ht="15">
+      <c r="A26" t="s" s="20">
         <v>12</v>
       </c>
       <c r="B26" s="20"/>
-      <c r="C26" s="21" t="s">
+      <c r="C26" t="s" s="21">
         <v>13</v>
       </c>
       <c r="D26" s="22"/>
@@ -1378,46 +1374,46 @@
       <c r="F26" s="22"/>
       <c r="G26" s="22"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="n">
+    <row r="27" spans="1:7" ht="15">
+      <c r="A27" s="25">
         <v>1</v>
       </c>
       <c r="B27" s="25"/>
-      <c r="C27" s="27" t="s">
+      <c r="C27" t="s" s="27">
         <v>18</v>
       </c>
-      <c r="D27" s="25" t="s">
+      <c r="D27" t="s" s="25">
         <v>19</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="25">
         <v>100</v>
       </c>
       <c r="F27" s="25"/>
       <c r="G27" s="25"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="n">
+    <row r="28" spans="1:7" ht="15">
+      <c r="A28" s="25">
         <v>2</v>
       </c>
       <c r="B28" s="25"/>
-      <c r="C28" s="27" t="s">
+      <c r="C28" t="s" s="27">
         <v>24</v>
       </c>
-      <c r="D28" s="25" t="s">
+      <c r="D28" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E28" s="25" t="n">
+      <c r="E28" s="25">
         <v>80</v>
       </c>
       <c r="F28" s="25"/>
       <c r="G28" s="25"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23" t="n">
+    <row r="29" spans="1:7" ht="15">
+      <c r="A29" s="23">
         <v>3</v>
       </c>
       <c r="B29" s="23"/>
-      <c r="C29" s="24" t="s">
+      <c r="C29" t="s" s="24">
         <v>36</v>
       </c>
       <c r="D29" s="25"/>
@@ -1425,27 +1421,27 @@
       <c r="F29" s="25"/>
       <c r="G29" s="25"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:7" ht="15">
       <c r="A30" s="23"/>
       <c r="B30" s="23"/>
-      <c r="C30" s="26" t="s">
+      <c r="C30" t="s" s="26">
         <v>37</v>
       </c>
-      <c r="D30" s="25" t="s">
+      <c r="D30" t="s" s="25">
         <v>16</v>
       </c>
-      <c r="E30" s="25" t="n">
+      <c r="E30" s="25">
         <v>250</v>
       </c>
       <c r="F30" s="25"/>
       <c r="G30" s="25"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+    <row r="31" spans="1:7" ht="15">
+      <c r="A31" t="s" s="20">
         <v>20</v>
       </c>
       <c r="B31" s="20"/>
-      <c r="C31" s="21" t="s">
+      <c r="C31" t="s" s="21">
         <v>21</v>
       </c>
       <c r="D31" s="22"/>
@@ -1453,82 +1449,82 @@
       <c r="F31" s="22"/>
       <c r="G31" s="22"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25" t="n">
+    <row r="32" spans="1:7" ht="15">
+      <c r="A32" s="25">
         <v>1</v>
       </c>
       <c r="B32" s="25"/>
-      <c r="C32" s="27" t="s">
+      <c r="C32" t="s" s="27">
         <v>22</v>
       </c>
-      <c r="D32" s="25" t="s">
+      <c r="D32" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E32" s="25" t="n">
+      <c r="E32" s="25">
         <v>150</v>
       </c>
       <c r="F32" s="25"/>
       <c r="G32" s="25"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="28" t="n">
+    <row r="33" spans="1:7" ht="15">
+      <c r="A33" s="28">
         <v>2</v>
       </c>
       <c r="B33" s="28"/>
-      <c r="C33" s="29" t="s">
+      <c r="C33" t="s" s="29">
         <v>31</v>
       </c>
-      <c r="D33" s="28" t="s">
+      <c r="D33" t="s" s="28">
         <v>26</v>
       </c>
-      <c r="E33" s="28" t="n">
+      <c r="E33" s="28">
         <v>5</v>
       </c>
       <c r="F33" s="28"/>
       <c r="G33" s="28"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="30" t="s">
+    <row r="34" spans="1:7" ht="15">
+      <c r="A34" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B34" s="30"/>
-      <c r="C34" s="31" t="s">
+      <c r="C34" t="s" s="31">
         <v>32</v>
       </c>
-      <c r="D34" s="30" t="s">
+      <c r="D34" t="s" s="30">
         <v>23</v>
       </c>
-      <c r="E34" s="30" t="n">
-        <f aca="false">E33*6</f>
+      <c r="E34" t="str" s="30">
+        <f>E33*6</f>
         <v>30</v>
       </c>
       <c r="F34" s="30"/>
       <c r="G34" s="30"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="30" t="s">
+    <row r="35" spans="1:7" ht="15">
+      <c r="A35" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B35" s="30"/>
-      <c r="C35" s="31" t="s">
+      <c r="C35" t="s" s="31">
         <v>38</v>
       </c>
-      <c r="D35" s="30" t="s">
+      <c r="D35" t="s" s="30">
         <v>26</v>
       </c>
-      <c r="E35" s="30" t="n">
-        <f aca="false">E33*1</f>
+      <c r="E35" t="str" s="30">
+        <f>E33*1</f>
         <v>5</v>
       </c>
       <c r="F35" s="30"/>
       <c r="G35" s="30"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="32" t="s">
+    <row r="36" spans="1:7" ht="15">
+      <c r="A36" t="s" s="32">
         <v>20</v>
       </c>
       <c r="B36" s="32"/>
-      <c r="C36" s="34" t="s">
+      <c r="C36" t="s" s="34">
         <v>39</v>
       </c>
       <c r="D36" s="34"/>
@@ -1536,8 +1532,8 @@
       <c r="F36" s="34"/>
       <c r="G36" s="35"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="s">
+    <row r="37" spans="1:7" ht="15">
+      <c r="A37" t="s" s="19">
         <v>40</v>
       </c>
       <c r="B37" s="19"/>
@@ -1547,12 +1543,12 @@
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
+    <row r="38" spans="1:7" ht="15">
+      <c r="A38" t="s" s="20">
         <v>12</v>
       </c>
       <c r="B38" s="20"/>
-      <c r="C38" s="21" t="s">
+      <c r="C38" t="s" s="21">
         <v>13</v>
       </c>
       <c r="D38" s="22"/>
@@ -1560,12 +1556,12 @@
       <c r="F38" s="22"/>
       <c r="G38" s="22"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="23" t="n">
+    <row r="39" spans="1:7" ht="15">
+      <c r="A39" s="23">
         <v>1</v>
       </c>
       <c r="B39" s="23"/>
-      <c r="C39" s="24" t="s">
+      <c r="C39" t="s" s="24">
         <v>14</v>
       </c>
       <c r="D39" s="25"/>
@@ -1573,27 +1569,27 @@
       <c r="F39" s="25"/>
       <c r="G39" s="25"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:7" ht="15">
       <c r="A40" s="23"/>
       <c r="B40" s="23"/>
-      <c r="C40" s="26" t="s">
+      <c r="C40" t="s" s="26">
         <v>15</v>
       </c>
-      <c r="D40" s="25" t="s">
+      <c r="D40" t="s" s="25">
         <v>16</v>
       </c>
-      <c r="E40" s="25" t="n">
+      <c r="E40" s="25">
         <v>500</v>
       </c>
       <c r="F40" s="25"/>
       <c r="G40" s="25"/>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="20" t="s">
+    <row r="41" spans="1:7" ht="15">
+      <c r="A41" t="s" s="20">
         <v>20</v>
       </c>
       <c r="B41" s="20"/>
-      <c r="C41" s="21" t="s">
+      <c r="C41" t="s" s="21">
         <v>21</v>
       </c>
       <c r="D41" s="22"/>
@@ -1601,116 +1597,116 @@
       <c r="F41" s="22"/>
       <c r="G41" s="22"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="25" t="n">
+    <row r="42" spans="1:7" ht="15">
+      <c r="A42" s="25">
         <v>1</v>
       </c>
       <c r="B42" s="25"/>
-      <c r="C42" s="27" t="s">
+      <c r="C42" t="s" s="27">
         <v>22</v>
       </c>
-      <c r="D42" s="25" t="s">
+      <c r="D42" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E42" s="25" t="n">
+      <c r="E42" s="25">
         <v>100</v>
       </c>
       <c r="F42" s="25"/>
       <c r="G42" s="25"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="28" t="n">
+    <row r="43" spans="1:7" ht="15">
+      <c r="A43" s="28">
         <v>2</v>
       </c>
       <c r="B43" s="28"/>
-      <c r="C43" s="29" t="s">
+      <c r="C43" t="s" s="29">
         <v>27</v>
       </c>
-      <c r="D43" s="28" t="s">
+      <c r="D43" t="s" s="28">
         <v>26</v>
       </c>
-      <c r="E43" s="28" t="n">
+      <c r="E43" s="28">
         <v>20</v>
       </c>
       <c r="F43" s="28"/>
       <c r="G43" s="28"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="30" t="s">
+    <row r="44" spans="1:7" ht="15">
+      <c r="A44" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B44" s="30"/>
-      <c r="C44" s="31" t="s">
+      <c r="C44" t="s" s="31">
         <v>30</v>
       </c>
-      <c r="D44" s="30" t="s">
+      <c r="D44" t="s" s="30">
         <v>26</v>
       </c>
-      <c r="E44" s="30" t="n">
-        <f aca="false">E43*1</f>
+      <c r="E44" t="str" s="30">
+        <f>E43*1</f>
         <v>20</v>
       </c>
       <c r="F44" s="30"/>
       <c r="G44" s="30"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="30" t="s">
+    <row r="45" spans="1:7" ht="15">
+      <c r="A45" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B45" s="30"/>
-      <c r="C45" s="31" t="s">
+      <c r="C45" t="s" s="31">
         <v>29</v>
       </c>
-      <c r="D45" s="30" t="s">
+      <c r="D45" t="s" s="30">
         <v>23</v>
       </c>
-      <c r="E45" s="30" t="n">
-        <f aca="false">E44*6</f>
+      <c r="E45" t="str" s="30">
+        <f>E44*6</f>
         <v>120</v>
       </c>
       <c r="F45" s="30"/>
       <c r="G45" s="30"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="25" t="n">
+    <row r="46" spans="1:7" ht="15">
+      <c r="A46" s="25">
         <v>3</v>
       </c>
       <c r="B46" s="25"/>
-      <c r="C46" s="27" t="s">
+      <c r="C46" t="s" s="27">
         <v>33</v>
       </c>
-      <c r="D46" s="25" t="s">
+      <c r="D46" t="s" s="25">
         <v>26</v>
       </c>
-      <c r="E46" s="25" t="n">
+      <c r="E46" s="25">
         <v>50</v>
       </c>
       <c r="F46" s="25"/>
       <c r="G46" s="25"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="25" t="n">
+    <row r="47" spans="1:7" ht="15">
+      <c r="A47" s="25">
         <v>4</v>
       </c>
       <c r="B47" s="25"/>
-      <c r="C47" s="27" t="s">
+      <c r="C47" t="s" s="27">
         <v>25</v>
       </c>
-      <c r="D47" s="25" t="s">
+      <c r="D47" t="s" s="25">
         <v>26</v>
       </c>
-      <c r="E47" s="25" t="n">
+      <c r="E47" s="25">
         <v>50</v>
       </c>
       <c r="F47" s="25"/>
       <c r="G47" s="25"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="32" t="s">
+    <row r="48" spans="1:7" ht="15">
+      <c r="A48" t="s" s="32">
         <v>41</v>
       </c>
       <c r="B48" s="32"/>
-      <c r="C48" s="34" t="s">
+      <c r="C48" t="s" s="34">
         <v>42</v>
       </c>
       <c r="D48" s="34"/>
@@ -1718,8 +1714,8 @@
       <c r="F48" s="34"/>
       <c r="G48" s="35"/>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="s">
+    <row r="49" spans="1:7" ht="15">
+      <c r="A49" t="s" s="19">
         <v>43</v>
       </c>
       <c r="B49" s="19"/>
@@ -1729,12 +1725,12 @@
       <c r="F49" s="19"/>
       <c r="G49" s="19"/>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="20" t="s">
+    <row r="50" spans="1:7" ht="15">
+      <c r="A50" t="s" s="20">
         <v>12</v>
       </c>
       <c r="B50" s="20"/>
-      <c r="C50" s="21" t="s">
+      <c r="C50" t="s" s="21">
         <v>13</v>
       </c>
       <c r="D50" s="22"/>
@@ -1742,29 +1738,29 @@
       <c r="F50" s="22"/>
       <c r="G50" s="22"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="25" t="n">
+    <row r="51" spans="1:7" ht="15">
+      <c r="A51" s="25">
         <v>1</v>
       </c>
       <c r="B51" s="25"/>
-      <c r="C51" s="27" t="s">
+      <c r="C51" t="s" s="27">
         <v>44</v>
       </c>
-      <c r="D51" s="25" t="s">
+      <c r="D51" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E51" s="25" t="n">
+      <c r="E51" s="25">
         <v>100</v>
       </c>
       <c r="F51" s="25"/>
       <c r="G51" s="25"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="23" t="n">
+    <row r="52" spans="1:7" ht="15">
+      <c r="A52" s="23">
         <v>2</v>
       </c>
       <c r="B52" s="23"/>
-      <c r="C52" s="24" t="s">
+      <c r="C52" t="s" s="24">
         <v>36</v>
       </c>
       <c r="D52" s="25"/>
@@ -1772,27 +1768,27 @@
       <c r="F52" s="25"/>
       <c r="G52" s="25"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:7" ht="15">
       <c r="A53" s="23"/>
       <c r="B53" s="23"/>
-      <c r="C53" s="26" t="s">
+      <c r="C53" t="s" s="26">
         <v>37</v>
       </c>
-      <c r="D53" s="25" t="s">
+      <c r="D53" t="s" s="25">
         <v>16</v>
       </c>
-      <c r="E53" s="25" t="n">
+      <c r="E53" s="25">
         <v>100</v>
       </c>
       <c r="F53" s="25"/>
       <c r="G53" s="25"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="23" t="n">
+    <row r="54" spans="1:7" ht="15">
+      <c r="A54" s="23">
         <v>3</v>
       </c>
       <c r="B54" s="23"/>
-      <c r="C54" s="24" t="s">
+      <c r="C54" t="s" s="24">
         <v>14</v>
       </c>
       <c r="D54" s="25"/>
@@ -1800,42 +1796,42 @@
       <c r="F54" s="25"/>
       <c r="G54" s="25"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:7" ht="15">
       <c r="A55" s="23"/>
       <c r="B55" s="23"/>
-      <c r="C55" s="26" t="s">
+      <c r="C55" t="s" s="26">
         <v>15</v>
       </c>
       <c r="D55" s="25"/>
-      <c r="E55" s="25" t="n">
+      <c r="E55" s="25">
         <v>250</v>
       </c>
       <c r="F55" s="25"/>
       <c r="G55" s="25"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="23" t="n">
+    <row r="56" spans="1:7" ht="15">
+      <c r="A56" s="23">
         <v>4</v>
       </c>
       <c r="B56" s="23"/>
-      <c r="C56" s="27" t="s">
+      <c r="C56" t="s" s="27">
         <v>17</v>
       </c>
-      <c r="D56" s="25" t="s">
+      <c r="D56" t="s" s="25">
         <v>16</v>
       </c>
-      <c r="E56" s="25" t="n">
+      <c r="E56" s="25">
         <v>500</v>
       </c>
       <c r="F56" s="25"/>
       <c r="G56" s="25"/>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="20" t="s">
+    <row r="57" spans="1:7" ht="15">
+      <c r="A57" t="s" s="20">
         <v>20</v>
       </c>
       <c r="B57" s="20"/>
-      <c r="C57" s="36" t="s">
+      <c r="C57" t="s" s="36">
         <v>21</v>
       </c>
       <c r="D57" s="22"/>
@@ -1843,52 +1839,52 @@
       <c r="F57" s="22"/>
       <c r="G57" s="22"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="25" t="n">
+    <row r="58" spans="1:7" ht="15">
+      <c r="A58" s="25">
         <v>1</v>
       </c>
       <c r="B58" s="25"/>
-      <c r="C58" s="27" t="s">
+      <c r="C58" t="s" s="27">
         <v>22</v>
       </c>
-      <c r="D58" s="25" t="s">
+      <c r="D58" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E58" s="25" t="n">
+      <c r="E58" s="25">
         <v>50</v>
       </c>
       <c r="F58" s="25"/>
       <c r="G58" s="25"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="25" t="n">
+    <row r="59" spans="1:7" ht="15">
+      <c r="A59" s="25">
         <v>2</v>
       </c>
       <c r="B59" s="25"/>
-      <c r="C59" s="27" t="s">
+      <c r="C59" t="s" s="27">
         <v>33</v>
       </c>
-      <c r="D59" s="25" t="s">
+      <c r="D59" t="s" s="25">
         <v>26</v>
       </c>
-      <c r="E59" s="25" t="n">
+      <c r="E59" s="25">
         <v>2</v>
       </c>
       <c r="F59" s="25"/>
       <c r="G59" s="25"/>
     </row>
-    <row r="60" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="28" t="n">
+    <row r="60" spans="1:15" ht="15" customFormat="1" s="37">
+      <c r="A60" s="28">
         <v>3</v>
       </c>
       <c r="B60" s="28"/>
-      <c r="C60" s="29" t="s">
+      <c r="C60" t="s" s="29">
         <v>31</v>
       </c>
-      <c r="D60" s="28" t="s">
+      <c r="D60" t="s" s="28">
         <v>26</v>
       </c>
-      <c r="E60" s="28" t="n">
+      <c r="E60" s="28">
         <v>10</v>
       </c>
       <c r="F60" s="28"/>
@@ -1900,21 +1896,21 @@
       <c r="L60" s="1"/>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
-      <c r="O60" s="0"/>
-    </row>
-    <row r="61" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="30" t="s">
+      <c r="O60"/>
+    </row>
+    <row r="61" spans="1:15" ht="15" customFormat="1" s="37">
+      <c r="A61" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B61" s="30"/>
-      <c r="C61" s="31" t="s">
+      <c r="C61" t="s" s="31">
         <v>32</v>
       </c>
-      <c r="D61" s="30" t="s">
+      <c r="D61" t="s" s="30">
         <v>23</v>
       </c>
-      <c r="E61" s="30" t="n">
-        <f aca="false">E60*6</f>
+      <c r="E61" t="str" s="30">
+        <f>E60*6</f>
         <v>60</v>
       </c>
       <c r="F61" s="30"/>
@@ -1926,38 +1922,38 @@
       <c r="L61" s="1"/>
       <c r="M61" s="1"/>
       <c r="N61" s="1"/>
-      <c r="O61" s="0"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="30" t="s">
+      <c r="O61"/>
+    </row>
+    <row r="62" spans="1:7" ht="15">
+      <c r="A62" t="s" s="30">
         <v>28</v>
       </c>
       <c r="B62" s="30"/>
-      <c r="C62" s="31" t="s">
+      <c r="C62" t="s" s="31">
         <v>38</v>
       </c>
-      <c r="D62" s="30" t="s">
+      <c r="D62" t="s" s="30">
         <v>26</v>
       </c>
-      <c r="E62" s="30" t="n">
-        <f aca="false">E60*1</f>
+      <c r="E62" t="str" s="30">
+        <f>E60*1</f>
         <v>10</v>
       </c>
       <c r="F62" s="30"/>
       <c r="G62" s="30"/>
     </row>
-    <row r="63" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="25" t="n">
+    <row r="63" spans="1:15" ht="15" customFormat="1" s="37">
+      <c r="A63" s="25">
         <v>4</v>
       </c>
       <c r="B63" s="25"/>
-      <c r="C63" s="27" t="s">
+      <c r="C63" t="s" s="27">
         <v>24</v>
       </c>
-      <c r="D63" s="25" t="s">
+      <c r="D63" t="s" s="25">
         <v>23</v>
       </c>
-      <c r="E63" s="25" t="n">
+      <c r="E63" s="25">
         <v>20</v>
       </c>
       <c r="F63" s="25"/>
@@ -1969,14 +1965,14 @@
       <c r="L63" s="1"/>
       <c r="M63" s="1"/>
       <c r="N63" s="1"/>
-      <c r="O63" s="0"/>
-    </row>
-    <row r="64" s="37" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="32" t="s">
+      <c r="O63"/>
+    </row>
+    <row r="64" spans="1:15" ht="15" customFormat="1" s="37">
+      <c r="A64" t="s" s="32">
         <v>45</v>
       </c>
       <c r="B64" s="32"/>
-      <c r="C64" s="34" t="s">
+      <c r="C64" t="s" s="34">
         <v>46</v>
       </c>
       <c r="D64" s="34"/>
@@ -1990,14 +1986,14 @@
       <c r="L64" s="1"/>
       <c r="M64" s="1"/>
       <c r="N64" s="1"/>
-      <c r="O64" s="0"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="38" t="s">
+      <c r="O64"/>
+    </row>
+    <row r="65" spans="1:7" ht="15">
+      <c r="A65" t="s" s="38">
         <v>47</v>
       </c>
       <c r="B65" s="38"/>
-      <c r="C65" s="39" t="s">
+      <c r="C65" t="s" s="39">
         <v>48</v>
       </c>
       <c r="D65" s="39"/>
@@ -2005,12 +2001,12 @@
       <c r="F65" s="39"/>
       <c r="G65" s="40"/>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="41" t="s">
+    <row r="66" spans="1:14" ht="15">
+      <c r="A66" t="s" s="41">
         <v>49</v>
       </c>
       <c r="B66" s="41"/>
-      <c r="C66" s="42" t="s">
+      <c r="C66" t="s" s="42">
         <v>50</v>
       </c>
       <c r="D66" s="42"/>
@@ -2025,12 +2021,12 @@
       <c r="M66" s="37"/>
       <c r="N66" s="37"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="44" t="s">
+    <row r="67" spans="1:14" ht="15">
+      <c r="A67" t="s" s="44">
         <v>51</v>
       </c>
       <c r="B67" s="44"/>
-      <c r="C67" s="45" t="s">
+      <c r="C67" t="s" s="45">
         <v>52</v>
       </c>
       <c r="D67" s="45"/>
@@ -2045,12 +2041,12 @@
       <c r="M67" s="37"/>
       <c r="N67" s="37"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="47" t="s">
+    <row r="68" spans="1:7" ht="15">
+      <c r="A68" t="s" s="47">
         <v>53</v>
       </c>
       <c r="B68" s="47"/>
-      <c r="C68" s="48" t="s">
+      <c r="C68" t="s" s="48">
         <v>54</v>
       </c>
       <c r="D68" s="48"/>
@@ -2058,7 +2054,7 @@
       <c r="F68" s="48"/>
       <c r="G68" s="49"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" spans="1:14" ht="15">
       <c r="A69" s="37"/>
       <c r="B69" s="37"/>
       <c r="C69" s="37"/>
@@ -2074,7 +2070,7 @@
       <c r="M69" s="37"/>
       <c r="N69" s="37"/>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" spans="1:14" ht="15">
       <c r="A70" s="37"/>
       <c r="B70" s="37"/>
       <c r="C70" s="37"/>
@@ -2115,12 +2111,310 @@
     <mergeCell ref="C67:F67"/>
     <mergeCell ref="C68:F68"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <phoneticPr fontId="1"/>
+  <printOptions horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" scale="100" orientation="portrait" fitToHeight="1" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr/>
+  <cols>
+    <col min="1" max="1" width="10.14" customWidth="1"/>
+    <col min="2" max="2" width="11.36" customWidth="1"/>
+    <col min="3" max="3" width="31.32" customWidth="1"/>
+    <col min="4" max="4" width="10.71" customWidth="1"/>
+    <col min="5" max="5" width="7.86" customWidth="1"/>
+    <col min="6" max="6" width="9.43" customWidth="1"/>
+    <col min="7" max="7" width="15.86" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="15" customHeight="1">
+      <c r="A1" s="23">
+        <v>1</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" t="s" s="24">
+        <v>14</v>
+      </c>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+    </row>
+    <row r="2" spans="1:7" ht="15" customHeight="1">
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" t="s" s="26">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s" s="25">
+        <v>16</v>
+      </c>
+      <c r="E2" s="25">
+        <v>950</v>
+      </c>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" customHeight="1">
+      <c r="A3" s="23">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23"/>
+      <c r="C3" t="s" s="27">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s" s="25">
+        <v>16</v>
+      </c>
+      <c r="E3" s="25">
+        <v>600</v>
+      </c>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" customHeight="1">
+      <c r="A4" s="23">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" t="s" s="27">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s" s="25">
+        <v>19</v>
+      </c>
+      <c r="E4" s="25">
+        <v>250</v>
+      </c>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+    </row>
+    <row r="5" spans="1:7" ht="15" customHeight="1">
+      <c r="A5" s="25">
+        <v>1</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" t="s" s="27">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s" s="25">
+        <v>23</v>
+      </c>
+      <c r="E5" s="25">
+        <v>599</v>
+      </c>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+    </row>
+    <row r="6" spans="1:7" ht="15" customHeight="1">
+      <c r="A6" s="25">
+        <v>2</v>
+      </c>
+      <c r="B6" s="25"/>
+      <c r="C6" t="s" s="27">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s" s="25">
+        <v>23</v>
+      </c>
+      <c r="E6" s="25">
+        <v>219</v>
+      </c>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+    </row>
+    <row r="7" spans="1:7" ht="15" customHeight="1">
+      <c r="A7" s="25">
+        <v>3</v>
+      </c>
+      <c r="B7" s="25"/>
+      <c r="C7" t="s" s="27">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s" s="25">
+        <v>26</v>
+      </c>
+      <c r="E7" s="25">
+        <v>52</v>
+      </c>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+    </row>
+    <row r="8" spans="1:7" ht="15" customHeight="1">
+      <c r="A8" s="28">
+        <v>4</v>
+      </c>
+      <c r="B8" s="28"/>
+      <c r="C8" t="s" s="29">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s" s="28">
+        <v>26</v>
+      </c>
+      <c r="E8" s="28">
+        <v>25</v>
+      </c>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+    </row>
+    <row r="9" spans="1:7" ht="15" customHeight="1">
+      <c r="A9" t="s" s="30">
+        <v>28</v>
+      </c>
+      <c r="B9" s="30"/>
+      <c r="C9" t="s" s="31">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s" s="30">
+        <v>23</v>
+      </c>
+      <c r="E9" s="30">
+        <v>150</v>
+      </c>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1">
+      <c r="A10" t="s" s="30">
+        <v>28</v>
+      </c>
+      <c r="B10" s="30"/>
+      <c r="C10" t="s" s="31">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s" s="30">
+        <v>26</v>
+      </c>
+      <c r="E10" s="30">
+        <v>25</v>
+      </c>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+    </row>
+    <row r="11" spans="1:7" ht="15" customHeight="1">
+      <c r="A11" s="28">
+        <v>5</v>
+      </c>
+      <c r="B11" s="28"/>
+      <c r="C11" t="s" s="29">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s" s="28">
+        <v>26</v>
+      </c>
+      <c r="E11" s="28">
+        <v>25</v>
+      </c>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+    </row>
+    <row r="12" spans="1:7" ht="15" customHeight="1">
+      <c r="A12" t="s" s="30">
+        <v>28</v>
+      </c>
+      <c r="B12" s="30"/>
+      <c r="C12" t="s" s="31">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s" s="30">
+        <v>23</v>
+      </c>
+      <c r="E12" s="30">
+        <v>150</v>
+      </c>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+    </row>
+    <row r="13" spans="1:7" ht="15" customHeight="1">
+      <c r="A13" t="s" s="30">
+        <v>28</v>
+      </c>
+      <c r="B13" s="30"/>
+      <c r="C13" t="s" s="31">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s" s="30">
+        <v>26</v>
+      </c>
+      <c r="E13" s="30">
+        <v>15</v>
+      </c>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+    </row>
+    <row r="14" spans="1:7" ht="15" customHeight="1">
+      <c r="A14" s="25">
+        <v>6</v>
+      </c>
+      <c r="B14" s="25"/>
+      <c r="C14" t="s" s="27">
+        <v>33</v>
+      </c>
+      <c r="D14" t="s" s="25">
+        <v>26</v>
+      </c>
+      <c r="E14" s="25">
+        <v>72</v>
+      </c>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+    </row>
+    <row r="15" spans="1:7" ht="15" customHeight="1">
+      <c r="A15" s="23">
+        <v>3</v>
+      </c>
+      <c r="B15" s="23"/>
+      <c r="C15" t="s" s="24">
+        <v>36</v>
+      </c>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+    </row>
+    <row r="16" spans="1:7" ht="15" customHeight="1">
+      <c r="A16" s="23"/>
+      <c r="B16" s="23"/>
+      <c r="C16" t="s" s="26">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s" s="25">
+        <v>16</v>
+      </c>
+      <c r="E16" s="25">
+        <v>350</v>
+      </c>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+    </row>
+    <row r="17" spans="1:7" ht="15" customHeight="1">
+      <c r="A17" s="25">
+        <v>1</v>
+      </c>
+      <c r="B17" s="25"/>
+      <c r="C17" t="s" s="27">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s" s="25">
+        <v>23</v>
+      </c>
+      <c r="E17" s="25">
+        <v>100</v>
+      </c>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A15:A16"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
 </file>
</xml_diff>